<commit_message>
feat(catalog): show how to read a workbook's other sheets and explain mixed cells
- An expanded Excel table says it holds the first sheet only and shows the
  read_xlsx query for another, by the name the workbook is registered under.
- A wrong sheet name gets the closest one suggested.
- A cell whose text doesn't fit its column's type, which read_xlsx takes
  from the first value, is named with its value and what to do.
- Opening an .xlsx by URL is covered by an end-to-end test.
</commit_message>
<xml_diff>
--- a/e2e/data/machines.xlsx
+++ b/e2e/data/machines.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet name="Sheet1" state="visible" sheetId="1" r:id="rId3"/>
+    <sheet name="Lines" state="visible" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -213,4 +214,53 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>hall</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(catalog): show how to read a workbook's other sheets and explain mixed cells (#179)
- An expanded Excel table says it holds the first sheet only and shows the
  read_xlsx query for another, by the name the workbook is registered under.
- A wrong sheet name gets the closest one suggested.
- A cell whose text doesn't fit its column's type, which read_xlsx takes
  from the first value, is named with its value and what to do.
- Opening an .xlsx by URL is covered by an end-to-end test.
</commit_message>
<xml_diff>
--- a/e2e/data/machines.xlsx
+++ b/e2e/data/machines.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet name="Sheet1" state="visible" sheetId="1" r:id="rId3"/>
+    <sheet name="Lines" state="visible" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -213,4 +214,53 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>hall</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>